<commit_message>
Cambios en el reporte 03/07/2025 -1
</commit_message>
<xml_diff>
--- a/documentos/static/documentos/files/Listado_de_entregables_plantilla.xlsx
+++ b/documentos/static/documentos/files/Listado_de_entregables_plantilla.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ingju\OneDrive - Cenyt ingenieros (1)\Python\Trazabilidad de documentos\Aplicacion_Documentos_Web\Junior 2\APLICACION_DOCUMENTOS\documentos\static\documentos\files\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://cenytingenieros-my.sharepoint.com/personal/desarrollo_cenyt_com_co/Documents/Python/Trazabilidad de documentos/Aplicacion_Documentos_Web/Deployment/APLICACION_DOCUMENTOS/documentos/static/documentos/files/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{B3019CE8-0051-43A6-8C39-A8F572780CAC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="12" documentId="8_{B3019CE8-0051-43A6-8C39-A8F572780CAC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{10D23DE8-898E-4E55-87F5-C9B88E5727CD}"/>
   <bookViews>
-    <workbookView xWindow="768" yWindow="768" windowWidth="21600" windowHeight="11232" xr2:uid="{36249E36-5DBF-4BFE-BFE2-F64AD3D03D29}"/>
+    <workbookView xWindow="28680" yWindow="-16380" windowWidth="16440" windowHeight="28320" xr2:uid="{36249E36-5DBF-4BFE-BFE2-F64AD3D03D29}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
   <si>
     <t>Proyecto:</t>
   </si>
@@ -50,19 +50,10 @@
     <t>DOCUMENTO / ACTIVIDAD</t>
   </si>
   <si>
-    <t>CEN1997</t>
+    <t>COD CLIENTE</t>
   </si>
   <si>
-    <t>Cen1997</t>
-  </si>
-  <si>
-    <t>11213213213</t>
-  </si>
-  <si>
-    <t>documento de prueba123</t>
-  </si>
-  <si>
-    <t>documento de prueba 2123124</t>
+    <t>documento de prueba 21231247</t>
   </si>
 </sst>
 </file>
@@ -133,7 +124,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="4">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -156,62 +147,41 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right/>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right/>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="49" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="2"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="2"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="2"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="2"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -552,69 +522,68 @@
   <cols>
     <col min="1" max="1" width="27.44140625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="45.109375" customWidth="1"/>
+    <col min="3" max="3" width="24.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A1" s="3" t="s">
+      <c r="A1" s="6" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="2"/>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A2" s="6" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" s="2"/>
+      <c r="D2" s="5"/>
+      <c r="E2" s="5"/>
+      <c r="F2" s="5"/>
+      <c r="G2" s="5"/>
+      <c r="H2" s="5"/>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A3" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B3" s="1" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A2" s="3" t="s">
-        <v>1</v>
+      <c r="C3" s="1" t="s">
+        <v>3</v>
       </c>
-      <c r="B2" s="1" t="s">
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A4" s="2"/>
+      <c r="B4" s="2"/>
+      <c r="C4" s="7"/>
+    </row>
+    <row r="5" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A5" s="3"/>
+      <c r="B5" s="3"/>
+      <c r="C5" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="C2" s="10"/>
-      <c r="D2" s="10"/>
-      <c r="E2" s="10"/>
-      <c r="F2" s="10"/>
-      <c r="G2" s="10"/>
-      <c r="H2" s="10"/>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A3" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="B3" s="2" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A4" s="4">
-        <v>1120580111</v>
-      </c>
-      <c r="B4" s="6" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A5" s="5" t="s">
-        <v>6</v>
-      </c>
-      <c r="B5" s="6" t="s">
-        <v>8</v>
-      </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A6" s="4"/>
-      <c r="B6" s="11"/>
+      <c r="A6" s="2"/>
+      <c r="B6" s="2"/>
+      <c r="C6" s="7"/>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A7" s="4"/>
-      <c r="B7" s="7"/>
+      <c r="A7" s="2"/>
+      <c r="B7" s="2"/>
+      <c r="C7" s="8"/>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A8" s="5"/>
-      <c r="B8" s="7"/>
+      <c r="A8" s="3"/>
+      <c r="B8" s="3"/>
+      <c r="C8" s="9"/>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A9" s="8"/>
-      <c r="B9" s="9"/>
+      <c r="A9" s="4"/>
+      <c r="B9" s="4"/>
+      <c r="C9" s="10"/>
     </row>
   </sheetData>
   <phoneticPr fontId="4" type="noConversion"/>

</xml_diff>

<commit_message>
Cambios en el reporte 03/07/2025 -2
</commit_message>
<xml_diff>
--- a/documentos/static/documentos/files/Listado_de_entregables_plantilla.xlsx
+++ b/documentos/static/documentos/files/Listado_de_entregables_plantilla.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ingju\OneDrive - Cenyt ingenieros (1)\Python\Trazabilidad de documentos\Aplicacion_Documentos_Web\Junior 2\APLICACION_DOCUMENTOS\documentos\static\documentos\files\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://cenytingenieros-my.sharepoint.com/personal/desarrollo_cenyt_com_co/Documents/Python/Trazabilidad de documentos/Aplicacion_Documentos_Web/Deployment/APLICACION_DOCUMENTOS/documentos/static/documentos/files/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{B3019CE8-0051-43A6-8C39-A8F572780CAC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="12" documentId="8_{B3019CE8-0051-43A6-8C39-A8F572780CAC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{10D23DE8-898E-4E55-87F5-C9B88E5727CD}"/>
   <bookViews>
-    <workbookView xWindow="768" yWindow="768" windowWidth="21600" windowHeight="11232" xr2:uid="{36249E36-5DBF-4BFE-BFE2-F64AD3D03D29}"/>
+    <workbookView xWindow="28680" yWindow="-16380" windowWidth="16440" windowHeight="28320" xr2:uid="{36249E36-5DBF-4BFE-BFE2-F64AD3D03D29}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
   <si>
     <t>Proyecto:</t>
   </si>
@@ -50,19 +50,10 @@
     <t>DOCUMENTO / ACTIVIDAD</t>
   </si>
   <si>
-    <t>CEN1997</t>
+    <t>COD CLIENTE</t>
   </si>
   <si>
-    <t>Cen1997</t>
-  </si>
-  <si>
-    <t>11213213213</t>
-  </si>
-  <si>
-    <t>documento de prueba123</t>
-  </si>
-  <si>
-    <t>documento de prueba 2123124</t>
+    <t>documento de prueba 21231247</t>
   </si>
 </sst>
 </file>
@@ -133,7 +124,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="4">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -156,62 +147,41 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right/>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right/>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="49" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="2"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="2"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="2"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="2"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -552,69 +522,68 @@
   <cols>
     <col min="1" max="1" width="27.44140625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="45.109375" customWidth="1"/>
+    <col min="3" max="3" width="24.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A1" s="3" t="s">
+      <c r="A1" s="6" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="2"/>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A2" s="6" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" s="2"/>
+      <c r="D2" s="5"/>
+      <c r="E2" s="5"/>
+      <c r="F2" s="5"/>
+      <c r="G2" s="5"/>
+      <c r="H2" s="5"/>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A3" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B3" s="1" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A2" s="3" t="s">
-        <v>1</v>
+      <c r="C3" s="1" t="s">
+        <v>3</v>
       </c>
-      <c r="B2" s="1" t="s">
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A4" s="2"/>
+      <c r="B4" s="2"/>
+      <c r="C4" s="7"/>
+    </row>
+    <row r="5" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A5" s="3"/>
+      <c r="B5" s="3"/>
+      <c r="C5" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="C2" s="10"/>
-      <c r="D2" s="10"/>
-      <c r="E2" s="10"/>
-      <c r="F2" s="10"/>
-      <c r="G2" s="10"/>
-      <c r="H2" s="10"/>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A3" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="B3" s="2" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A4" s="4">
-        <v>1120580111</v>
-      </c>
-      <c r="B4" s="6" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A5" s="5" t="s">
-        <v>6</v>
-      </c>
-      <c r="B5" s="6" t="s">
-        <v>8</v>
-      </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A6" s="4"/>
-      <c r="B6" s="11"/>
+      <c r="A6" s="2"/>
+      <c r="B6" s="2"/>
+      <c r="C6" s="7"/>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A7" s="4"/>
-      <c r="B7" s="7"/>
+      <c r="A7" s="2"/>
+      <c r="B7" s="2"/>
+      <c r="C7" s="8"/>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A8" s="5"/>
-      <c r="B8" s="7"/>
+      <c r="A8" s="3"/>
+      <c r="B8" s="3"/>
+      <c r="C8" s="9"/>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A9" s="8"/>
-      <c r="B9" s="9"/>
+      <c r="A9" s="4"/>
+      <c r="B9" s="4"/>
+      <c r="C9" s="10"/>
     </row>
   </sheetData>
   <phoneticPr fontId="4" type="noConversion"/>

</xml_diff>

<commit_message>
Nueva funcion de backup
</commit_message>
<xml_diff>
--- a/documentos/static/documentos/files/Listado_de_entregables_plantilla.xlsx
+++ b/documentos/static/documentos/files/Listado_de_entregables_plantilla.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://cenytingenieros-my.sharepoint.com/personal/desarrollo_cenyt_com_co/Documents/Python/Trazabilidad de documentos/Aplicacion_Documentos_Web/Deployment/APLICACION_DOCUMENTOS/documentos/static/documentos/files/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://cenytingenieros-my.sharepoint.com/personal/desarrollo_cenyt_com_co/Documents/Python/Trazabilidad de documentos/Aplicacion_Documentos_Web/Junior 2/APLICACION_DOCUMENTOS/documentos/static/documentos/files/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="12" documentId="8_{B3019CE8-0051-43A6-8C39-A8F572780CAC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{10D23DE8-898E-4E55-87F5-C9B88E5727CD}"/>
+  <xr:revisionPtr revIDLastSave="13" documentId="8_{B3019CE8-0051-43A6-8C39-A8F572780CAC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{09BBD8B8-F968-47BD-B7A4-799495A8D691}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-16380" windowWidth="16440" windowHeight="28320" xr2:uid="{36249E36-5DBF-4BFE-BFE2-F64AD3D03D29}"/>
+    <workbookView xWindow="2688" yWindow="2688" windowWidth="17280" windowHeight="8880" xr2:uid="{36249E36-5DBF-4BFE-BFE2-F64AD3D03D29}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5" uniqueCount="5">
   <si>
     <t>Proyecto:</t>
   </si>
@@ -51,9 +51,6 @@
   </si>
   <si>
     <t>COD CLIENTE</t>
-  </si>
-  <si>
-    <t>documento de prueba 21231247</t>
   </si>
 </sst>
 </file>
@@ -558,12 +555,10 @@
       <c r="B4" s="2"/>
       <c r="C4" s="7"/>
     </row>
-    <row r="5" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A5" s="3"/>
       <c r="B5" s="3"/>
-      <c r="C5" s="7" t="s">
-        <v>5</v>
-      </c>
+      <c r="C5" s="7"/>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A6" s="2"/>

</xml_diff>